<commit_message>
chore: auto-add Htmlbl to 前端开发
</commit_message>
<xml_diff>
--- a/tools.xlsx
+++ b/tools.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,37 @@
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>前端开发</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Htmlbl</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://github.com/mountopjh/Htmlbl</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>